<commit_message>
Cambios en la tabla relacional entrega 2
</commit_message>
<xml_diff>
--- a/Entrega_2/Modelo_Relacional/Modelo_Relacional.xlsx
+++ b/Entrega_2/Modelo_Relacional/Modelo_Relacional.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="172">
   <si>
     <t>Empresa, sedes y oferta de servicios</t>
   </si>
@@ -51,13 +51,10 @@
     <t>Nit_Empresa</t>
   </si>
   <si>
-    <t>bigint</t>
+    <t>int</t>
   </si>
   <si>
     <t>Cod_Sede</t>
-  </si>
-  <si>
-    <t>int</t>
   </si>
   <si>
     <t>Cod_Plan</t>
@@ -1176,7 +1173,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="75">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1195,6 +1192,9 @@
     </xf>
     <xf borderId="5" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="5" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1248,6 +1248,9 @@
     <xf borderId="17" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf borderId="17" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="18" fillId="5" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1263,9 +1266,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf borderId="21" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="21" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="21" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="21" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="22" fillId="6" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1333,6 +1339,9 @@
     </xf>
     <xf borderId="37" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="37" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="37" fillId="0" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1689,167 +1698,167 @@
       <c r="G6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="9" t="s">
-        <v>12</v>
+      <c r="H6" s="10" t="s">
+        <v>10</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>8</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="L6" s="9" t="s">
         <v>12</v>
+      </c>
+      <c r="L6" s="10" t="s">
+        <v>10</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>8</v>
       </c>
       <c r="O6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="P6" s="10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="18.0" customHeight="1">
+      <c r="B7" s="11"/>
+      <c r="C7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="P6" s="9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" ht="18.0" customHeight="1">
-      <c r="B7" s="10"/>
-      <c r="C7" s="8" t="s">
+      <c r="D7" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="F7" s="11"/>
+      <c r="G7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="8" t="s">
+      <c r="H7" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" s="11"/>
+      <c r="K7" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J7" s="10"/>
-      <c r="K7" s="8" t="s">
+      <c r="L7" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="N7" s="11"/>
+      <c r="O7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="N7" s="10"/>
-      <c r="O7" s="8" t="s">
+      <c r="P7" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="11"/>
+      <c r="C8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="P7" s="9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="10"/>
-      <c r="C8" s="8" t="s">
+      <c r="D8" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="10"/>
-      <c r="G8" s="8" t="s">
+      <c r="H8" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J8" s="11"/>
+      <c r="K8" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" s="10"/>
-      <c r="K8" s="8" t="s">
+      <c r="L8" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="N8" s="11"/>
+      <c r="O8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="L8" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="N8" s="10"/>
-      <c r="O8" s="8" t="s">
+      <c r="P8" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="11"/>
+      <c r="C9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="P8" s="9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="10"/>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" s="11"/>
+      <c r="K9" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="H9" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="10"/>
-      <c r="K9" s="8" t="s">
+      <c r="L9" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="N9" s="11"/>
+      <c r="O9" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="L9" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="N9" s="10"/>
-      <c r="O9" s="8" t="s">
+      <c r="P9" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" ht="21.75" customHeight="1">
+      <c r="F10" s="11"/>
+      <c r="G10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="P9" s="9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" ht="21.75" customHeight="1">
-      <c r="F10" s="10"/>
-      <c r="G10" s="8" t="s">
+      <c r="H10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="J10" s="11"/>
+      <c r="K10" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="H10" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="J10" s="10"/>
-      <c r="K10" s="8" t="s">
+      <c r="L10" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="L10" s="9" t="s">
+      <c r="N10" s="11"/>
+      <c r="O10" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="N10" s="10"/>
-      <c r="O10" s="8" t="s">
+      <c r="P10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="P10" s="9" t="s">
+    </row>
+    <row r="11">
+      <c r="F11" s="11"/>
+      <c r="G11" s="8" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="F11" s="10"/>
-      <c r="G11" s="8" t="s">
+      <c r="H11" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J11" s="11"/>
+      <c r="K11" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="H11" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="J11" s="10"/>
-      <c r="K11" s="8" t="s">
+      <c r="L11" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="N11" s="11"/>
+      <c r="O11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="N11" s="10"/>
-      <c r="O11" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="P11" s="9" t="s">
-        <v>16</v>
+      <c r="P11" s="10" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="12" ht="19.5" customHeight="1">
       <c r="F12" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>9</v>
@@ -1858,7 +1867,7 @@
         <v>10</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K12" s="8" t="s">
         <v>9</v>
@@ -1869,22 +1878,22 @@
     </row>
     <row r="15">
       <c r="B15" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="5"/>
       <c r="F15" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="5"/>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="K15" s="13"/>
+      <c r="L15" s="14"/>
+      <c r="N15" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="K15" s="12"/>
-      <c r="L15" s="13"/>
-      <c r="N15" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="O15" s="4"/>
       <c r="P15" s="5"/>
@@ -1908,13 +1917,13 @@
       <c r="H16" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="J16" s="14" t="s">
+      <c r="J16" s="15" t="s">
         <v>5</v>
       </c>
       <c r="K16" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="L16" s="15" t="s">
+      <c r="L16" s="16" t="s">
         <v>7</v>
       </c>
       <c r="N16" s="6" t="s">
@@ -1932,200 +1941,200 @@
         <v>8</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>12</v>
+        <v>40</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>10</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>8</v>
       </c>
       <c r="G17" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="J17" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="K17" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="H17" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="J17" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="K17" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="L17" s="17" t="s">
-        <v>12</v>
+      <c r="L17" s="18" t="s">
+        <v>10</v>
       </c>
       <c r="N17" s="7" t="s">
         <v>8</v>
       </c>
       <c r="O17" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="P17" s="10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="11"/>
+      <c r="C18" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="P17" s="9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="10"/>
-      <c r="C18" s="8" t="s">
+      <c r="D18" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="11"/>
+      <c r="G18" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F18" s="10"/>
-      <c r="G18" s="8" t="s">
+      <c r="H18" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J18" s="19"/>
+      <c r="K18" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H18" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J18" s="18"/>
-      <c r="K18" s="8" t="s">
+      <c r="L18" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="L18" s="17" t="s">
+      <c r="N18" s="11"/>
+      <c r="O18" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="N18" s="10"/>
-      <c r="O18" s="8" t="s">
+      <c r="P18" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="11"/>
+      <c r="C19" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="P18" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="10"/>
-      <c r="C19" s="8" t="s">
+      <c r="D19" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="11"/>
+      <c r="G19" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="10"/>
-      <c r="G19" s="8" t="s">
+      <c r="H19" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J19" s="19"/>
+      <c r="K19" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="H19" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J19" s="18"/>
-      <c r="K19" s="8" t="s">
+      <c r="L19" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="N19" s="11"/>
+      <c r="O19" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="L19" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="N19" s="10"/>
-      <c r="O19" s="8" t="s">
+      <c r="P19" s="10" t="s">
         <v>53</v>
-      </c>
-      <c r="P19" s="9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" s="10"/>
+      <c r="D20" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="11"/>
       <c r="G20" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J20" s="19"/>
+      <c r="K20" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="H20" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J20" s="18"/>
-      <c r="K20" s="8" t="s">
+      <c r="L20" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="N20" s="11"/>
+      <c r="O20" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="L20" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="N20" s="10"/>
-      <c r="O20" s="8" t="s">
+      <c r="P20" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="F21" s="11"/>
+      <c r="G21" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="P20" s="9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="F21" s="10"/>
-      <c r="G21" s="8" t="s">
+      <c r="H21" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="H21" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J21" s="19" t="s">
+      <c r="K21" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="L21" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="N21" s="11"/>
+      <c r="O21" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="K21" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="L21" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="N21" s="10"/>
-      <c r="O21" s="8" t="s">
+      <c r="P21" s="10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="F22" s="11"/>
+      <c r="G22" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="P21" s="9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="F22" s="10"/>
-      <c r="G22" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>48</v>
+      <c r="H22" s="10" t="s">
+        <v>47</v>
       </c>
       <c r="N22" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O22" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="P22" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="P22" s="10" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="23" ht="19.5" customHeight="1">
       <c r="F23" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>12</v>
+        <v>40</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>10</v>
       </c>
       <c r="N23" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O23" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="P23" s="9" t="s">
-        <v>12</v>
+        <v>40</v>
+      </c>
+      <c r="P23" s="10" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="N24" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O24" s="8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P24" s="9" t="s">
         <v>10</v>
@@ -2136,7 +2145,7 @@
     <row r="27" ht="15.75" customHeight="1"/>
     <row r="28" ht="15.75" customHeight="1">
       <c r="B28" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -2156,25 +2165,25 @@
     <row r="29" ht="15.75" customHeight="1"/>
     <row r="30" ht="15.75" customHeight="1">
       <c r="B30" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="5"/>
       <c r="F30" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="5"/>
       <c r="J30" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K30" s="4"/>
       <c r="L30" s="5"/>
-      <c r="N30" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="O30" s="12"/>
-      <c r="P30" s="13"/>
+      <c r="N30" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="O30" s="13"/>
+      <c r="P30" s="14"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="B31" s="6" t="s">
@@ -2204,13 +2213,13 @@
       <c r="L31" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="N31" s="14" t="s">
+      <c r="N31" s="15" t="s">
         <v>5</v>
       </c>
       <c r="O31" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="P31" s="15" t="s">
+      <c r="P31" s="16" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2219,7 +2228,7 @@
         <v>8</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D32" s="9" t="s">
         <v>10</v>
@@ -2228,177 +2237,177 @@
         <v>8</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>12</v>
+        <v>68</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>10</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>8</v>
       </c>
       <c r="K32" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="L32" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="N32" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="O32" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="L32" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="N32" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="O32" s="8" t="s">
+      <c r="P32" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="P32" s="17" t="s">
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="B33" s="11"/>
+      <c r="C33" s="8" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="B33" s="10"/>
-      <c r="C33" s="8" t="s">
+      <c r="D33" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F33" s="11"/>
+      <c r="G33" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="D33" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F33" s="10"/>
-      <c r="G33" s="8" t="s">
+      <c r="H33" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J33" s="11"/>
+      <c r="K33" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="H33" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="J33" s="10"/>
-      <c r="K33" s="8" t="s">
+      <c r="L33" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="N33" s="19"/>
+      <c r="O33" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="L33" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="N33" s="18"/>
-      <c r="O33" s="8" t="s">
+      <c r="P33" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="B34" s="11"/>
+      <c r="C34" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="P33" s="17" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="B34" s="10"/>
-      <c r="C34" s="8" t="s">
+      <c r="D34" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" s="11"/>
+      <c r="G34" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F34" s="10"/>
-      <c r="G34" s="8" t="s">
+      <c r="H34" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="J34" s="11"/>
+      <c r="K34" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="H34" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="J34" s="10"/>
-      <c r="K34" s="8" t="s">
+      <c r="L34" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="O34" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="P34" s="18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="B35" s="11"/>
+      <c r="C35" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="L34" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="N34" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="O34" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="P34" s="17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="B35" s="10"/>
-      <c r="C35" s="8" t="s">
+      <c r="D35" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F35" s="11"/>
+      <c r="G35" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D35" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F35" s="10"/>
-      <c r="G35" s="8" t="s">
+      <c r="H35" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J35" s="11"/>
+      <c r="K35" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="H35" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J35" s="10"/>
-      <c r="K35" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="L35" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="N35" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="O35" s="20" t="s">
+      <c r="L35" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="N35" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="O35" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="P35" s="21" t="s">
-        <v>12</v>
+      <c r="P35" s="22" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="36" ht="21.75" customHeight="1">
       <c r="B36" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C36" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="H36" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="J36" s="11"/>
+      <c r="K36" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="D36" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F36" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="G36" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="J36" s="10"/>
-      <c r="K36" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="L36" s="9" t="s">
-        <v>32</v>
+      <c r="L36" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="F37" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H37" s="9" t="s">
         <v>12</v>
       </c>
+      <c r="H37" s="10" t="s">
+        <v>10</v>
+      </c>
       <c r="J37" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K37" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="L37" s="9" t="s">
-        <v>12</v>
+        <v>68</v>
+      </c>
+      <c r="L37" s="10" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="38" ht="19.5" customHeight="1">
       <c r="J38" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K38" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L38" s="9" t="s">
         <v>10</v>
@@ -2407,138 +2416,138 @@
     <row r="39" ht="15.75" customHeight="1"/>
     <row r="40" ht="15.75" customHeight="1"/>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="C41" s="24"/>
+      <c r="D41" s="25"/>
+      <c r="F41" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="C41" s="23"/>
-      <c r="D41" s="24"/>
-      <c r="F41" s="22" t="s">
+      <c r="G41" s="24"/>
+      <c r="H41" s="25"/>
+      <c r="J41" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="G41" s="23"/>
-      <c r="H41" s="24"/>
-      <c r="J41" s="22" t="s">
+      <c r="K41" s="24"/>
+      <c r="L41" s="25"/>
+      <c r="N41" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="K41" s="23"/>
-      <c r="L41" s="24"/>
-      <c r="N41" s="22" t="s">
+      <c r="O41" s="24"/>
+      <c r="P41" s="25"/>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="B42" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F42" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="G42" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="H42" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="J42" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="K42" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="L42" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="N42" s="26" t="s">
+        <v>5</v>
+      </c>
+      <c r="O42" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="P42" s="26" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="B43" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="O41" s="23"/>
-      <c r="P41" s="24"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
-      <c r="B42" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="C42" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="D42" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="F42" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="G42" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="H42" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="J42" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="K42" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="L42" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="N42" s="25" t="s">
-        <v>5</v>
-      </c>
-      <c r="O42" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="P42" s="25" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
-      <c r="B43" s="26" t="s">
+      <c r="D43" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="C43" s="27" t="s">
+      <c r="G43" s="28" t="s">
         <v>90</v>
       </c>
-      <c r="D43" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="F43" s="26" t="s">
+      <c r="H43" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="J43" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="G43" s="27" t="s">
+      <c r="K43" s="28" t="s">
         <v>91</v>
       </c>
-      <c r="H43" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="J43" s="26" t="s">
+      <c r="L43" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="N43" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="K43" s="27" t="s">
+      <c r="O43" s="28" t="s">
         <v>92</v>
       </c>
-      <c r="L43" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="N43" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="O43" s="27" t="s">
-        <v>93</v>
-      </c>
-      <c r="P43" s="28" t="s">
-        <v>16</v>
+      <c r="P43" s="29" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="B44" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="C44" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="D44" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="F44" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="G44" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="H44" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="J44" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="K44" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="L44" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="N44" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="O44" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="P44" s="28" t="s">
+      <c r="B44" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="C44" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="D44" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="G44" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="H44" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="J44" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="K44" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="L44" s="30" t="s">
+        <v>10</v>
+      </c>
+      <c r="N44" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="O44" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="P44" s="30" t="s">
         <v>10</v>
       </c>
     </row>
@@ -2547,7 +2556,7 @@
     <row r="47" ht="15.75" customHeight="1"/>
     <row r="48" ht="15.75" customHeight="1">
       <c r="B48" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -2567,20 +2576,20 @@
     <row r="49" ht="19.5" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1">
       <c r="B50" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C50" s="4"/>
       <c r="D50" s="5"/>
-      <c r="F50" s="29" t="s">
+      <c r="F50" s="31" t="s">
+        <v>95</v>
+      </c>
+      <c r="G50" s="32"/>
+      <c r="H50" s="33"/>
+      <c r="J50" s="31" t="s">
         <v>96</v>
       </c>
-      <c r="G50" s="30"/>
-      <c r="H50" s="31"/>
-      <c r="J50" s="29" t="s">
-        <v>97</v>
-      </c>
-      <c r="K50" s="30"/>
-      <c r="L50" s="31"/>
+      <c r="K50" s="32"/>
+      <c r="L50" s="33"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="B51" s="6" t="s">
@@ -2592,22 +2601,22 @@
       <c r="D51" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F51" s="32" t="s">
+      <c r="F51" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="G51" s="32" t="s">
+      <c r="G51" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="H51" s="32" t="s">
+      <c r="H51" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="J51" s="32" t="s">
+      <c r="J51" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="K51" s="32" t="s">
+      <c r="K51" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="L51" s="32" t="s">
+      <c r="L51" s="34" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2616,100 +2625,100 @@
         <v>8</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D52" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F52" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="G52" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="H52" s="35" t="s">
-        <v>10</v>
-      </c>
-      <c r="J52" s="33" t="s">
-        <v>59</v>
-      </c>
-      <c r="K52" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="L52" s="35" t="s">
+      <c r="F52" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="G52" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="H52" s="37" t="s">
+        <v>10</v>
+      </c>
+      <c r="J52" s="35" t="s">
+        <v>58</v>
+      </c>
+      <c r="K52" s="36" t="s">
+        <v>84</v>
+      </c>
+      <c r="L52" s="37" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="B53" s="10"/>
+      <c r="B53" s="11"/>
       <c r="C53" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F53" s="38"/>
+      <c r="G53" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="D53" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F53" s="36"/>
-      <c r="G53" s="34" t="s">
+      <c r="H53" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="J53" s="38"/>
+      <c r="K53" s="36" t="s">
         <v>99</v>
       </c>
-      <c r="H53" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="J53" s="36"/>
-      <c r="K53" s="34" t="s">
+      <c r="L53" s="39" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1">
+      <c r="B54" s="11"/>
+      <c r="C54" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="L53" s="35" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="54" ht="15.75" customHeight="1">
-      <c r="B54" s="10"/>
-      <c r="C54" s="8" t="s">
+      <c r="D54" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1">
+      <c r="B55" s="11"/>
+      <c r="C55" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="D54" s="9" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="55" ht="15.75" customHeight="1">
-      <c r="B55" s="10"/>
-      <c r="C55" s="8" t="s">
+      <c r="D55" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="56" ht="21.75" customHeight="1">
+      <c r="B56" s="11"/>
+      <c r="C56" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D55" s="9" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="56" ht="21.75" customHeight="1">
-      <c r="B56" s="10"/>
-      <c r="C56" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D56" s="9" t="s">
-        <v>30</v>
+      <c r="D56" s="10" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="B57" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D57" s="9" t="s">
-        <v>12</v>
+      <c r="D57" s="10" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="58" ht="19.5" customHeight="1">
       <c r="B58" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="D58" s="9" t="s">
-        <v>12</v>
+        <v>82</v>
+      </c>
+      <c r="D58" s="10" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1"/>
@@ -2717,7 +2726,7 @@
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1">
       <c r="B62" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" s="2"/>
@@ -2736,247 +2745,247 @@
     </row>
     <row r="63" ht="15.75" customHeight="1"/>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="B64" s="37" t="s">
+      <c r="B64" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C64" s="41"/>
+      <c r="D64" s="42"/>
+      <c r="F64" s="43" t="s">
         <v>105</v>
       </c>
-      <c r="C64" s="38"/>
-      <c r="D64" s="39"/>
-      <c r="F64" s="40" t="s">
+      <c r="G64" s="44"/>
+      <c r="H64" s="45"/>
+      <c r="J64" s="40" t="s">
         <v>106</v>
       </c>
-      <c r="G64" s="41"/>
-      <c r="H64" s="42"/>
-      <c r="J64" s="37" t="s">
+      <c r="K64" s="41"/>
+      <c r="L64" s="42"/>
+      <c r="N64" s="40" t="s">
         <v>107</v>
       </c>
-      <c r="K64" s="38"/>
-      <c r="L64" s="39"/>
-      <c r="N64" s="37" t="s">
+      <c r="O64" s="41"/>
+      <c r="P64" s="42"/>
+    </row>
+    <row r="65" ht="15.75" customHeight="1">
+      <c r="B65" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="D65" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="F65" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="G65" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="H65" s="48" t="s">
+        <v>7</v>
+      </c>
+      <c r="J65" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="K65" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="L65" s="46" t="s">
+        <v>7</v>
+      </c>
+      <c r="N65" s="46" t="s">
+        <v>5</v>
+      </c>
+      <c r="O65" s="46" t="s">
+        <v>6</v>
+      </c>
+      <c r="P65" s="46" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66" ht="15.75" customHeight="1">
+      <c r="B66" s="49" t="s">
+        <v>8</v>
+      </c>
+      <c r="C66" s="50" t="s">
+        <v>82</v>
+      </c>
+      <c r="D66" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" s="52" t="s">
+        <v>8</v>
+      </c>
+      <c r="G66" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="O64" s="38"/>
-      <c r="P64" s="39"/>
-    </row>
-    <row r="65" ht="15.75" customHeight="1">
-      <c r="B65" s="43" t="s">
-        <v>5</v>
-      </c>
-      <c r="C65" s="43" t="s">
-        <v>6</v>
-      </c>
-      <c r="D65" s="43" t="s">
-        <v>7</v>
-      </c>
-      <c r="F65" s="44" t="s">
-        <v>5</v>
-      </c>
-      <c r="G65" s="43" t="s">
-        <v>6</v>
-      </c>
-      <c r="H65" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="J65" s="43" t="s">
-        <v>5</v>
-      </c>
-      <c r="K65" s="43" t="s">
-        <v>6</v>
-      </c>
-      <c r="L65" s="43" t="s">
-        <v>7</v>
-      </c>
-      <c r="N65" s="43" t="s">
-        <v>5</v>
-      </c>
-      <c r="O65" s="43" t="s">
-        <v>6</v>
-      </c>
-      <c r="P65" s="43" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="66" ht="15.75" customHeight="1">
-      <c r="B66" s="46" t="s">
+      <c r="H66" s="53" t="s">
+        <v>71</v>
+      </c>
+      <c r="J66" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="C66" s="47" t="s">
-        <v>83</v>
-      </c>
-      <c r="D66" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="F66" s="49" t="s">
+      <c r="K66" s="50" t="s">
+        <v>109</v>
+      </c>
+      <c r="L66" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="N66" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="G66" s="47" t="s">
+      <c r="O66" s="50" t="s">
+        <v>110</v>
+      </c>
+      <c r="P66" s="51" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="67" ht="15.75" customHeight="1">
+      <c r="B67" s="54"/>
+      <c r="C67" s="50" t="s">
+        <v>111</v>
+      </c>
+      <c r="D67" s="51" t="s">
+        <v>15</v>
+      </c>
+      <c r="F67" s="55"/>
+      <c r="G67" s="50" t="s">
+        <v>112</v>
+      </c>
+      <c r="H67" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="J67" s="54"/>
+      <c r="K67" s="50" t="s">
+        <v>113</v>
+      </c>
+      <c r="L67" s="51" t="s">
+        <v>15</v>
+      </c>
+      <c r="N67" s="54"/>
+      <c r="O67" s="50" t="s">
+        <v>114</v>
+      </c>
+      <c r="P67" s="51" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68" ht="15.75" customHeight="1">
+      <c r="B68" s="54"/>
+      <c r="C68" s="50" t="s">
+        <v>115</v>
+      </c>
+      <c r="D68" s="51" t="s">
+        <v>15</v>
+      </c>
+      <c r="F68" s="55"/>
+      <c r="G68" s="50" t="s">
+        <v>116</v>
+      </c>
+      <c r="H68" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="J68" s="54"/>
+      <c r="K68" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="L68" s="51" t="s">
+        <v>15</v>
+      </c>
+      <c r="N68" s="54"/>
+      <c r="O68" s="50" t="s">
+        <v>118</v>
+      </c>
+      <c r="P68" s="51" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69" ht="15.75" customHeight="1">
+      <c r="B69" s="54"/>
+      <c r="C69" s="50" t="s">
+        <v>119</v>
+      </c>
+      <c r="D69" s="51" t="s">
+        <v>31</v>
+      </c>
+      <c r="F69" s="55"/>
+      <c r="G69" s="50" t="s">
+        <v>120</v>
+      </c>
+      <c r="H69" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="J69" s="54"/>
+      <c r="K69" s="50" t="s">
+        <v>121</v>
+      </c>
+      <c r="L69" s="51" t="s">
+        <v>15</v>
+      </c>
+      <c r="N69" s="54"/>
+      <c r="O69" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="P69" s="51" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="70" ht="21.75" customHeight="1">
+      <c r="B70" s="54"/>
+      <c r="C70" s="50" t="s">
+        <v>123</v>
+      </c>
+      <c r="D70" s="51" t="s">
+        <v>47</v>
+      </c>
+      <c r="F70" s="56" t="s">
+        <v>58</v>
+      </c>
+      <c r="G70" s="57" t="s">
+        <v>82</v>
+      </c>
+      <c r="H70" s="58" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" ht="15.75" customHeight="1">
+      <c r="B71" s="54"/>
+      <c r="C71" s="50" t="s">
+        <v>124</v>
+      </c>
+      <c r="D71" s="51" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="72" ht="19.5" customHeight="1">
+      <c r="B72" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="C72" s="50" t="s">
         <v>109</v>
       </c>
-      <c r="H66" s="50" t="s">
-        <v>72</v>
-      </c>
-      <c r="J66" s="46" t="s">
-        <v>8</v>
-      </c>
-      <c r="K66" s="47" t="s">
-        <v>110</v>
-      </c>
-      <c r="L66" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="N66" s="46" t="s">
-        <v>8</v>
-      </c>
-      <c r="O66" s="47" t="s">
-        <v>111</v>
-      </c>
-      <c r="P66" s="48" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="67" ht="15.75" customHeight="1">
-      <c r="B67" s="51"/>
-      <c r="C67" s="47" t="s">
-        <v>112</v>
-      </c>
-      <c r="D67" s="48" t="s">
-        <v>16</v>
-      </c>
-      <c r="F67" s="52"/>
-      <c r="G67" s="47" t="s">
-        <v>113</v>
-      </c>
-      <c r="H67" s="50" t="s">
-        <v>16</v>
-      </c>
-      <c r="J67" s="51"/>
-      <c r="K67" s="47" t="s">
-        <v>114</v>
-      </c>
-      <c r="L67" s="48" t="s">
-        <v>16</v>
-      </c>
-      <c r="N67" s="51"/>
-      <c r="O67" s="47" t="s">
-        <v>115</v>
-      </c>
-      <c r="P67" s="48" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="68" ht="15.75" customHeight="1">
-      <c r="B68" s="51"/>
-      <c r="C68" s="47" t="s">
-        <v>116</v>
-      </c>
-      <c r="D68" s="48" t="s">
-        <v>16</v>
-      </c>
-      <c r="F68" s="52"/>
-      <c r="G68" s="47" t="s">
-        <v>117</v>
-      </c>
-      <c r="H68" s="50" t="s">
-        <v>16</v>
-      </c>
-      <c r="J68" s="51"/>
-      <c r="K68" s="47" t="s">
-        <v>118</v>
-      </c>
-      <c r="L68" s="48" t="s">
-        <v>16</v>
-      </c>
-      <c r="N68" s="51"/>
-      <c r="O68" s="47" t="s">
-        <v>119</v>
-      </c>
-      <c r="P68" s="48" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="69" ht="15.75" customHeight="1">
-      <c r="B69" s="51"/>
-      <c r="C69" s="47" t="s">
-        <v>120</v>
-      </c>
-      <c r="D69" s="48" t="s">
-        <v>32</v>
-      </c>
-      <c r="F69" s="52"/>
-      <c r="G69" s="47" t="s">
-        <v>121</v>
-      </c>
-      <c r="H69" s="50" t="s">
-        <v>16</v>
-      </c>
-      <c r="J69" s="51"/>
-      <c r="K69" s="47" t="s">
-        <v>122</v>
-      </c>
-      <c r="L69" s="48" t="s">
-        <v>16</v>
-      </c>
-      <c r="N69" s="51"/>
-      <c r="O69" s="47" t="s">
-        <v>123</v>
-      </c>
-      <c r="P69" s="48" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="70" ht="21.75" customHeight="1">
-      <c r="B70" s="51"/>
-      <c r="C70" s="47" t="s">
-        <v>124</v>
-      </c>
-      <c r="D70" s="48" t="s">
-        <v>48</v>
-      </c>
-      <c r="F70" s="53" t="s">
-        <v>59</v>
-      </c>
-      <c r="G70" s="54" t="s">
-        <v>83</v>
-      </c>
-      <c r="H70" s="55" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="71" ht="15.75" customHeight="1">
-      <c r="B71" s="51"/>
-      <c r="C71" s="47" t="s">
+      <c r="D72" s="51" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73" ht="15.75" customHeight="1">
+      <c r="B73" s="54"/>
+      <c r="C73" s="50" t="s">
         <v>125</v>
       </c>
-      <c r="D71" s="48" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="72" ht="19.5" customHeight="1">
-      <c r="B72" s="46" t="s">
-        <v>36</v>
-      </c>
-      <c r="C72" s="47" t="s">
-        <v>110</v>
-      </c>
-      <c r="D72" s="48" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="73" ht="15.75" customHeight="1">
-      <c r="B73" s="51"/>
-      <c r="C73" s="47" t="s">
+      <c r="D73" s="51" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="74" ht="15.75" customHeight="1">
+      <c r="B74" s="54"/>
+      <c r="C74" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="D73" s="48" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="74" ht="15.75" customHeight="1">
-      <c r="B74" s="51"/>
-      <c r="C74" s="47" t="s">
-        <v>127</v>
-      </c>
-      <c r="D74" s="48" t="s">
-        <v>48</v>
+      <c r="D74" s="51" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1"/>
@@ -2984,7 +2993,7 @@
     <row r="77" ht="15.75" customHeight="1"/>
     <row r="78" ht="15.75" customHeight="1">
       <c r="B78" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" s="2"/>
@@ -3003,220 +3012,220 @@
     </row>
     <row r="79" ht="15.75" customHeight="1"/>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="B80" s="56" t="s">
+      <c r="B80" s="59" t="s">
+        <v>128</v>
+      </c>
+      <c r="C80" s="60"/>
+      <c r="D80" s="61"/>
+      <c r="F80" s="59" t="s">
         <v>129</v>
       </c>
-      <c r="C80" s="57"/>
-      <c r="D80" s="58"/>
-      <c r="F80" s="56" t="s">
+      <c r="G80" s="60"/>
+      <c r="H80" s="61"/>
+      <c r="J80" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="G80" s="57"/>
-      <c r="H80" s="58"/>
-      <c r="J80" s="56" t="s">
+      <c r="K80" s="60"/>
+      <c r="L80" s="61"/>
+      <c r="N80" s="59" t="s">
         <v>131</v>
       </c>
-      <c r="K80" s="57"/>
-      <c r="L80" s="58"/>
-      <c r="N80" s="56" t="s">
+      <c r="O80" s="60"/>
+      <c r="P80" s="61"/>
+    </row>
+    <row r="81" ht="15.75" customHeight="1">
+      <c r="B81" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="C81" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="D81" s="62" t="s">
+        <v>7</v>
+      </c>
+      <c r="F81" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="G81" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="H81" s="62" t="s">
+        <v>7</v>
+      </c>
+      <c r="J81" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="K81" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="L81" s="62" t="s">
+        <v>7</v>
+      </c>
+      <c r="N81" s="62" t="s">
+        <v>5</v>
+      </c>
+      <c r="O81" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="P81" s="62" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="82" ht="15.75" customHeight="1">
+      <c r="B82" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="C82" s="64" t="s">
+        <v>11</v>
+      </c>
+      <c r="D82" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="F82" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="G82" s="64" t="s">
+        <v>13</v>
+      </c>
+      <c r="H82" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="J82" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="K82" s="64" t="s">
+        <v>13</v>
+      </c>
+      <c r="L82" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="N82" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="O82" s="64" t="s">
+        <v>43</v>
+      </c>
+      <c r="P82" s="65" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" ht="15.75" customHeight="1">
+      <c r="B83" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="C83" s="64" t="s">
+        <v>12</v>
+      </c>
+      <c r="D83" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="F83" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="G83" s="64" t="s">
+        <v>12</v>
+      </c>
+      <c r="H83" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="J83" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="K83" s="64" t="s">
+        <v>11</v>
+      </c>
+      <c r="L83" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="N83" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="O83" s="64" t="s">
+        <v>67</v>
+      </c>
+      <c r="P83" s="66" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="84" ht="15.75" customHeight="1">
+      <c r="F84" s="67"/>
+      <c r="G84" s="64" t="s">
         <v>132</v>
       </c>
-      <c r="O80" s="57"/>
-      <c r="P80" s="58"/>
-    </row>
-    <row r="81" ht="15.75" customHeight="1">
-      <c r="B81" s="59" t="s">
-        <v>5</v>
-      </c>
-      <c r="C81" s="59" t="s">
-        <v>6</v>
-      </c>
-      <c r="D81" s="59" t="s">
-        <v>7</v>
-      </c>
-      <c r="F81" s="59" t="s">
-        <v>5</v>
-      </c>
-      <c r="G81" s="59" t="s">
-        <v>6</v>
-      </c>
-      <c r="H81" s="59" t="s">
-        <v>7</v>
-      </c>
-      <c r="J81" s="59" t="s">
-        <v>5</v>
-      </c>
-      <c r="K81" s="59" t="s">
-        <v>6</v>
-      </c>
-      <c r="L81" s="59" t="s">
-        <v>7</v>
-      </c>
-      <c r="N81" s="59" t="s">
-        <v>5</v>
-      </c>
-      <c r="O81" s="59" t="s">
-        <v>6</v>
-      </c>
-      <c r="P81" s="59" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="82" ht="15.75" customHeight="1">
-      <c r="B82" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="C82" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="D82" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="F82" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="G82" s="61" t="s">
-        <v>14</v>
-      </c>
-      <c r="H82" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="J82" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="K82" s="61" t="s">
-        <v>14</v>
-      </c>
-      <c r="L82" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="N82" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="O82" s="61" t="s">
-        <v>44</v>
-      </c>
-      <c r="P82" s="62" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="83" ht="15.75" customHeight="1">
-      <c r="B83" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="C83" s="61" t="s">
-        <v>13</v>
-      </c>
-      <c r="D83" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="F83" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="G83" s="61" t="s">
-        <v>13</v>
-      </c>
-      <c r="H83" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="J83" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="K83" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="L83" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="N83" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="O83" s="61" t="s">
-        <v>68</v>
-      </c>
-      <c r="P83" s="62" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="84" ht="15.75" customHeight="1">
-      <c r="F84" s="63"/>
-      <c r="G84" s="61" t="s">
+      <c r="H84" s="65" t="s">
+        <v>10</v>
+      </c>
+      <c r="J84" s="67"/>
+      <c r="K84" s="64" t="s">
         <v>133</v>
       </c>
-      <c r="H84" s="62" t="s">
-        <v>12</v>
-      </c>
-      <c r="J84" s="63"/>
-      <c r="K84" s="61" t="s">
+      <c r="L84" s="65" t="s">
+        <v>15</v>
+      </c>
+      <c r="N84" s="67"/>
+      <c r="O84" s="64" t="s">
         <v>134</v>
       </c>
-      <c r="L84" s="62" t="s">
-        <v>16</v>
-      </c>
-      <c r="N84" s="63"/>
-      <c r="O84" s="61" t="s">
+      <c r="P84" s="65" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="85" ht="15.75" customHeight="1">
+      <c r="F85" s="67"/>
+      <c r="G85" s="64" t="s">
         <v>135</v>
       </c>
-      <c r="P84" s="62" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="85" ht="15.75" customHeight="1">
-      <c r="F85" s="63"/>
-      <c r="G85" s="61" t="s">
+      <c r="H85" s="65" t="s">
+        <v>29</v>
+      </c>
+      <c r="N85" s="67"/>
+      <c r="O85" s="64" t="s">
         <v>136</v>
       </c>
-      <c r="H85" s="62" t="s">
-        <v>30</v>
-      </c>
-      <c r="N85" s="63"/>
-      <c r="O85" s="61" t="s">
-        <v>137</v>
-      </c>
-      <c r="P85" s="62" t="s">
-        <v>32</v>
+      <c r="P85" s="65" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="86" ht="21.75" customHeight="1"/>
     <row r="87" ht="15.75" customHeight="1"/>
     <row r="88" ht="19.5" customHeight="1">
-      <c r="B88" s="56" t="s">
-        <v>138</v>
-      </c>
-      <c r="C88" s="57"/>
-      <c r="D88" s="58"/>
+      <c r="B88" s="59" t="s">
+        <v>137</v>
+      </c>
+      <c r="C88" s="60"/>
+      <c r="D88" s="61"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="B89" s="59" t="s">
+      <c r="B89" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="C89" s="59" t="s">
+      <c r="C89" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="D89" s="59" t="s">
+      <c r="D89" s="62" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="B90" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="C90" s="61" t="s">
+      <c r="B90" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="C90" s="64" t="s">
+        <v>109</v>
+      </c>
+      <c r="D90" s="65" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="91" ht="15.75" customHeight="1">
+      <c r="B91" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="C91" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="D90" s="62" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="91" ht="15.75" customHeight="1">
-      <c r="B91" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="C91" s="61" t="s">
-        <v>111</v>
-      </c>
-      <c r="D91" s="62" t="s">
-        <v>12</v>
+      <c r="D91" s="65" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1"/>
@@ -3224,43 +3233,43 @@
     <row r="94" ht="15.75" customHeight="1"/>
     <row r="95" ht="15.75" customHeight="1"/>
     <row r="96" ht="19.5" customHeight="1">
-      <c r="B96" s="56" t="s">
-        <v>138</v>
-      </c>
-      <c r="C96" s="57"/>
-      <c r="D96" s="58"/>
+      <c r="B96" s="59" t="s">
+        <v>137</v>
+      </c>
+      <c r="C96" s="60"/>
+      <c r="D96" s="61"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="B97" s="59" t="s">
+      <c r="B97" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="C97" s="59" t="s">
+      <c r="C97" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="D97" s="59" t="s">
+      <c r="D97" s="62" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1">
-      <c r="B98" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="C98" s="61" t="s">
+      <c r="B98" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="C98" s="64" t="s">
+        <v>109</v>
+      </c>
+      <c r="D98" s="65" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="99" ht="15.75" customHeight="1">
+      <c r="B99" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="C99" s="64" t="s">
         <v>110</v>
       </c>
-      <c r="D98" s="62" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="99" ht="15.75" customHeight="1">
-      <c r="B99" s="60" t="s">
-        <v>59</v>
-      </c>
-      <c r="C99" s="61" t="s">
-        <v>111</v>
-      </c>
-      <c r="D99" s="62" t="s">
-        <v>12</v>
+      <c r="D99" s="65" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="100" ht="15.75" customHeight="1"/>
@@ -4166,35 +4175,35 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="J15:L15"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="J41:L41"/>
+    <mergeCell ref="N41:P41"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="J30:L30"/>
+    <mergeCell ref="N30:P30"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="F41:H41"/>
+    <mergeCell ref="B80:D80"/>
+    <mergeCell ref="F80:H80"/>
+    <mergeCell ref="J80:L80"/>
+    <mergeCell ref="N80:P80"/>
+    <mergeCell ref="B88:D88"/>
+    <mergeCell ref="B96:D96"/>
     <mergeCell ref="B50:D50"/>
+    <mergeCell ref="F50:H50"/>
+    <mergeCell ref="J50:L50"/>
     <mergeCell ref="B64:D64"/>
     <mergeCell ref="F64:H64"/>
     <mergeCell ref="J64:L64"/>
-    <mergeCell ref="B96:D96"/>
-    <mergeCell ref="B80:D80"/>
-    <mergeCell ref="F80:H80"/>
-    <mergeCell ref="B88:D88"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="N4:P4"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="F15:H15"/>
     <mergeCell ref="N64:P64"/>
-    <mergeCell ref="J15:L15"/>
-    <mergeCell ref="N15:P15"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="J30:L30"/>
-    <mergeCell ref="N30:P30"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="F41:H41"/>
-    <mergeCell ref="J41:L41"/>
-    <mergeCell ref="N41:P41"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="J50:L50"/>
-    <mergeCell ref="J80:L80"/>
-    <mergeCell ref="N80:P80"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -4219,615 +4228,615 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="64" t="s">
+      <c r="B2" s="68" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" s="68" t="s">
         <v>139</v>
       </c>
-      <c r="C2" s="64" t="s">
+      <c r="D2" s="68" t="s">
         <v>140</v>
       </c>
-      <c r="D2" s="64" t="s">
+      <c r="E2" s="68" t="s">
         <v>141</v>
       </c>
-      <c r="E2" s="64" t="s">
+      <c r="F2" s="68" t="s">
         <v>142</v>
       </c>
-      <c r="F2" s="64" t="s">
+    </row>
+    <row r="3">
+      <c r="B3" s="69" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="70" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="70" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" s="70" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="70" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="3">
-      <c r="B3" s="65" t="s">
+    <row r="4">
+      <c r="B4" s="69" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="70" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="70" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="70" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="70" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="69" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="70" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="66" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="66" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" s="66" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" s="66" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="65" t="s">
+      <c r="E5" s="70" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="70" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="69" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="70" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="70" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="70" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="70" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="69" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="70" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="70" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="70" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="70" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="69" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="70" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="70" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="69" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="70" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="70" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="70" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="70" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="69" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="70" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="70" t="s">
+        <v>95</v>
+      </c>
+      <c r="E10" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="70" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="69" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="D11" s="70" t="s">
+        <v>104</v>
+      </c>
+      <c r="E11" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="F11" s="70" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="69" t="s">
+        <v>64</v>
+      </c>
+      <c r="C12" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" s="70" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="70" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="69" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="70" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="66" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="66" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="66" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="66" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="65" t="s">
-        <v>37</v>
-      </c>
-      <c r="C5" s="66" t="s">
+      <c r="E13" s="70" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="70" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="69" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="F14" s="70" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="69" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="70" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="70" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="69" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="70" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" s="70" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="70" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="69" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="70" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="66" t="s">
+      <c r="D17" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="66" t="s">
+      <c r="E17" s="70" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="66" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="65" t="s">
-        <v>38</v>
-      </c>
-      <c r="C6" s="66" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" s="66" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="66" t="s">
-        <v>41</v>
-      </c>
-      <c r="F6" s="66" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="65" t="s">
+      <c r="F17" s="70" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="71" t="s">
+        <v>85</v>
+      </c>
+      <c r="C18" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" s="70" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="F18" s="70" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="71" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="70" t="s">
+        <v>63</v>
+      </c>
+      <c r="E19" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="F19" s="70" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="71" t="s">
+        <v>87</v>
+      </c>
+      <c r="C20" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" s="70" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="F20" s="70" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="B21" s="71" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="70" t="s">
+        <v>63</v>
+      </c>
+      <c r="E21" s="70" t="s">
+        <v>67</v>
+      </c>
+      <c r="F21" s="70" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="B22" s="69" t="s">
+        <v>94</v>
+      </c>
+      <c r="C22" s="70" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="70" t="s">
+        <v>2</v>
+      </c>
+      <c r="E22" s="70" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="70" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="B23" s="69" t="s">
+        <v>94</v>
+      </c>
+      <c r="C23" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="D23" s="70" t="s">
+        <v>104</v>
+      </c>
+      <c r="E23" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="F23" s="70" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="B24" s="72" t="s">
+        <v>95</v>
+      </c>
+      <c r="C24" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="D24" s="70" t="s">
+        <v>94</v>
+      </c>
+      <c r="E24" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="F24" s="70" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="B25" s="72" t="s">
+        <v>96</v>
+      </c>
+      <c r="C25" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="D25" s="70" t="s">
+        <v>94</v>
+      </c>
+      <c r="E25" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="F25" s="70" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="B26" s="73" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="70" t="s">
+        <v>109</v>
+      </c>
+      <c r="D26" s="70" t="s">
+        <v>106</v>
+      </c>
+      <c r="E26" s="70" t="s">
+        <v>109</v>
+      </c>
+      <c r="F26" s="70" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="B27" s="73" t="s">
+        <v>105</v>
+      </c>
+      <c r="C27" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="D27" s="70" t="s">
+        <v>104</v>
+      </c>
+      <c r="E27" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="F27" s="70" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="B28" s="74" t="s">
+        <v>128</v>
+      </c>
+      <c r="C28" s="70" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="70" t="s">
+        <v>2</v>
+      </c>
+      <c r="E28" s="70" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="70" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="B29" s="74" t="s">
+        <v>128</v>
+      </c>
+      <c r="C29" s="70" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="E29" s="70" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="70" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="B30" s="74" t="s">
+        <v>129</v>
+      </c>
+      <c r="C30" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="70" t="s">
+        <v>4</v>
+      </c>
+      <c r="E30" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" s="70" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="B31" s="74" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" s="70" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="70" t="s">
+        <v>3</v>
+      </c>
+      <c r="E31" s="70" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" s="70" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="B32" s="74" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="70" t="s">
+        <v>4</v>
+      </c>
+      <c r="E32" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="70" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="B33" s="74" t="s">
+        <v>130</v>
+      </c>
+      <c r="C33" s="70" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="70" t="s">
+        <v>2</v>
+      </c>
+      <c r="E33" s="70" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="70" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="B34" s="74" t="s">
+        <v>131</v>
+      </c>
+      <c r="C34" s="70" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="66" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" s="66" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" s="66" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="66" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="65" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="66" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="66" t="s">
-        <v>4</v>
-      </c>
-      <c r="E8" s="66" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="66" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="65" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="66" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="66" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="66" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" s="66" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="65" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="66" t="s">
-        <v>62</v>
-      </c>
-      <c r="D10" s="66" t="s">
-        <v>96</v>
-      </c>
-      <c r="E10" s="66" t="s">
-        <v>85</v>
-      </c>
-      <c r="F10" s="66" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="65" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" s="66" t="s">
-        <v>83</v>
-      </c>
-      <c r="D11" s="66" t="s">
-        <v>105</v>
-      </c>
-      <c r="E11" s="66" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" s="66" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="65" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="D12" s="66" t="s">
-        <v>64</v>
-      </c>
-      <c r="E12" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="F12" s="66" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="65" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" s="66" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" s="66" t="s">
-        <v>3</v>
-      </c>
-      <c r="E13" s="66" t="s">
-        <v>13</v>
-      </c>
-      <c r="F13" s="66" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="65" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="66" t="s">
-        <v>69</v>
-      </c>
-      <c r="D14" s="66" t="s">
-        <v>65</v>
-      </c>
-      <c r="E14" s="66" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="66" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="65" t="s">
-        <v>66</v>
-      </c>
-      <c r="C15" s="66" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="66" t="s">
-        <v>95</v>
-      </c>
-      <c r="E15" s="66" t="s">
-        <v>85</v>
-      </c>
-      <c r="F15" s="66" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="65" t="s">
+      <c r="E34" s="70" t="s">
+        <v>43</v>
+      </c>
+      <c r="F34" s="70" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="B35" s="74" t="s">
+        <v>131</v>
+      </c>
+      <c r="C35" s="70" t="s">
         <v>67</v>
       </c>
-      <c r="C16" s="66" t="s">
-        <v>69</v>
-      </c>
-      <c r="D16" s="66" t="s">
-        <v>65</v>
-      </c>
-      <c r="E16" s="66" t="s">
-        <v>69</v>
-      </c>
-      <c r="F16" s="66" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="65" t="s">
+      <c r="D35" s="70" t="s">
+        <v>63</v>
+      </c>
+      <c r="E35" s="70" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="66" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="66" t="s">
-        <v>2</v>
-      </c>
-      <c r="E17" s="66" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="66" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="67" t="s">
-        <v>86</v>
-      </c>
-      <c r="C18" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="D18" s="66" t="s">
-        <v>64</v>
-      </c>
-      <c r="E18" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="F18" s="66" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="67" t="s">
-        <v>87</v>
-      </c>
-      <c r="C19" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="D19" s="66" t="s">
-        <v>64</v>
-      </c>
-      <c r="E19" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="F19" s="66" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="67" t="s">
-        <v>88</v>
-      </c>
-      <c r="C20" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="D20" s="66" t="s">
-        <v>64</v>
-      </c>
-      <c r="E20" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="F20" s="66" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="B21" s="67" t="s">
-        <v>89</v>
-      </c>
-      <c r="C21" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="D21" s="66" t="s">
-        <v>64</v>
-      </c>
-      <c r="E21" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="F21" s="66" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="B22" s="65" t="s">
-        <v>95</v>
-      </c>
-      <c r="C22" s="66" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="66" t="s">
-        <v>2</v>
-      </c>
-      <c r="E22" s="66" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="66" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="B23" s="65" t="s">
-        <v>95</v>
-      </c>
-      <c r="C23" s="66" t="s">
-        <v>83</v>
-      </c>
-      <c r="D23" s="66" t="s">
-        <v>105</v>
-      </c>
-      <c r="E23" s="66" t="s">
-        <v>83</v>
-      </c>
-      <c r="F23" s="66" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="B24" s="68" t="s">
-        <v>96</v>
-      </c>
-      <c r="C24" s="66" t="s">
-        <v>85</v>
-      </c>
-      <c r="D24" s="66" t="s">
-        <v>95</v>
-      </c>
-      <c r="E24" s="66" t="s">
-        <v>85</v>
-      </c>
-      <c r="F24" s="66" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="B25" s="68" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" s="66" t="s">
-        <v>85</v>
-      </c>
-      <c r="D25" s="66" t="s">
-        <v>95</v>
-      </c>
-      <c r="E25" s="66" t="s">
-        <v>85</v>
-      </c>
-      <c r="F25" s="66" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="B26" s="69" t="s">
-        <v>105</v>
-      </c>
-      <c r="C26" s="66" t="s">
+      <c r="F35" s="70" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="B36" s="74" t="s">
+        <v>137</v>
+      </c>
+      <c r="C36" s="70" t="s">
+        <v>109</v>
+      </c>
+      <c r="D36" s="70" t="s">
+        <v>106</v>
+      </c>
+      <c r="E36" s="70" t="s">
+        <v>109</v>
+      </c>
+      <c r="F36" s="70" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="B37" s="74" t="s">
+        <v>137</v>
+      </c>
+      <c r="C37" s="70" t="s">
         <v>110</v>
       </c>
-      <c r="D26" s="66" t="s">
+      <c r="D37" s="70" t="s">
         <v>107</v>
       </c>
-      <c r="E26" s="66" t="s">
+      <c r="E37" s="70" t="s">
         <v>110</v>
       </c>
-      <c r="F26" s="66" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="B27" s="69" t="s">
-        <v>106</v>
-      </c>
-      <c r="C27" s="66" t="s">
-        <v>83</v>
-      </c>
-      <c r="D27" s="66" t="s">
-        <v>105</v>
-      </c>
-      <c r="E27" s="66" t="s">
-        <v>83</v>
-      </c>
-      <c r="F27" s="66" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="B28" s="70" t="s">
-        <v>129</v>
-      </c>
-      <c r="C28" s="66" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="66" t="s">
-        <v>2</v>
-      </c>
-      <c r="E28" s="66" t="s">
-        <v>11</v>
-      </c>
-      <c r="F28" s="66" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="B29" s="70" t="s">
-        <v>129</v>
-      </c>
-      <c r="C29" s="66" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="66" t="s">
-        <v>3</v>
-      </c>
-      <c r="E29" s="66" t="s">
-        <v>13</v>
-      </c>
-      <c r="F29" s="66" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="B30" s="70" t="s">
-        <v>130</v>
-      </c>
-      <c r="C30" s="66" t="s">
-        <v>14</v>
-      </c>
-      <c r="D30" s="66" t="s">
-        <v>4</v>
-      </c>
-      <c r="E30" s="66" t="s">
-        <v>14</v>
-      </c>
-      <c r="F30" s="66" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="B31" s="70" t="s">
-        <v>130</v>
-      </c>
-      <c r="C31" s="66" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" s="66" t="s">
-        <v>3</v>
-      </c>
-      <c r="E31" s="66" t="s">
-        <v>13</v>
-      </c>
-      <c r="F31" s="66" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="B32" s="70" t="s">
-        <v>131</v>
-      </c>
-      <c r="C32" s="66" t="s">
-        <v>14</v>
-      </c>
-      <c r="D32" s="66" t="s">
-        <v>4</v>
-      </c>
-      <c r="E32" s="66" t="s">
-        <v>14</v>
-      </c>
-      <c r="F32" s="66" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="B33" s="70" t="s">
-        <v>131</v>
-      </c>
-      <c r="C33" s="66" t="s">
-        <v>11</v>
-      </c>
-      <c r="D33" s="66" t="s">
-        <v>2</v>
-      </c>
-      <c r="E33" s="66" t="s">
-        <v>11</v>
-      </c>
-      <c r="F33" s="66" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="B34" s="70" t="s">
-        <v>132</v>
-      </c>
-      <c r="C34" s="66" t="s">
-        <v>44</v>
-      </c>
-      <c r="D34" s="66" t="s">
-        <v>40</v>
-      </c>
-      <c r="E34" s="66" t="s">
-        <v>44</v>
-      </c>
-      <c r="F34" s="66" t="s">
+      <c r="F37" s="70" t="s">
         <v>171</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="B35" s="70" t="s">
-        <v>132</v>
-      </c>
-      <c r="C35" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="D35" s="66" t="s">
-        <v>64</v>
-      </c>
-      <c r="E35" s="66" t="s">
-        <v>68</v>
-      </c>
-      <c r="F35" s="66" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="B36" s="70" t="s">
-        <v>138</v>
-      </c>
-      <c r="C36" s="66" t="s">
-        <v>110</v>
-      </c>
-      <c r="D36" s="66" t="s">
-        <v>107</v>
-      </c>
-      <c r="E36" s="66" t="s">
-        <v>110</v>
-      </c>
-      <c r="F36" s="66" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="B37" s="70" t="s">
-        <v>138</v>
-      </c>
-      <c r="C37" s="66" t="s">
-        <v>111</v>
-      </c>
-      <c r="D37" s="66" t="s">
-        <v>108</v>
-      </c>
-      <c r="E37" s="66" t="s">
-        <v>111</v>
-      </c>
-      <c r="F37" s="66" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1"/>

</xml_diff>